<commit_message>
added confirmed cases map
</commit_message>
<xml_diff>
--- a/src/R/translations.xlsx
+++ b/src/R/translations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5aee5c5b004427f/Documents/mr-risk-assessment/src/R/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="8_{4649215D-82E5-4B27-B6A2-F5C81FA3C8C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC46462B-165B-4FAF-858F-A03536C628BE}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{132F1232-AAEB-42DF-9114-B0462C5F7248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{278938BD-8EEF-4A72-B5CF-EA4A40E5C537}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{41A3C097-9B5C-484B-88DA-6A6C7D19F152}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{41A3C097-9B5C-484B-88DA-6A6C7D19F152}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORT" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="MSG" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">DASHBOARD!$A$1:$E$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">DASHBOARD!$A$1:$E$196</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">MSG!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">QA_REPORT!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">REPORT!$A$1:$E$170</definedName>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2285" uniqueCount="1672">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2310" uniqueCount="1681">
   <si>
     <t>LABEL</t>
   </si>
@@ -7245,78 +7245,24 @@
     <t>Fechar</t>
   </si>
   <si>
-    <t>silent_mun_lab</t>
-  </si>
-  <si>
-    <t>Municipios silenciosos</t>
-  </si>
-  <si>
-    <t>Silent municipalities</t>
-  </si>
-  <si>
-    <t>Municípios silenciosos</t>
-  </si>
-  <si>
-    <t>Municipalités silencieuses</t>
-  </si>
-  <si>
-    <t>silent_mun_legend</t>
-  </si>
-  <si>
     <t>Reporta casos sospechosos</t>
   </si>
   <si>
     <t>Signale des cas suspects</t>
   </si>
   <si>
-    <t>silent_mun_infobox_text</t>
-  </si>
-  <si>
     <t>title_figure_3f</t>
   </si>
   <si>
-    <t>silent_mun_lab_pct</t>
-  </si>
-  <si>
-    <t>Notifica casos suspeitos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reports suspected cases </t>
-  </si>
-  <si>
     <t>Equipo capacitado en los últimos 2 años</t>
   </si>
   <si>
     <t>Areas subnacionales con un equipo que ha sido capacitado en respuesta a brotes en los últimos 2 años</t>
   </si>
   <si>
-    <t>Municipios que no reportan casos sospechosos</t>
-  </si>
-  <si>
-    <t>Número de municipios que no reportan casos sospechosos</t>
-  </si>
-  <si>
     <t>Presencia de un equipo capacitado en los últimos 2 años (Puntaje)</t>
   </si>
   <si>
-    <t>Municipalities that do not report suspected cases</t>
-  </si>
-  <si>
-    <t>Number of municipalities that do not report suspected cases</t>
-  </si>
-  <si>
-    <t>Municípios que não reportam casos suspeitos</t>
-  </si>
-  <si>
-    <t>Número de municípios que não reportam casos suspeitos</t>
-  </si>
-  <si>
-    <t>Municipalités qui ne signalent pas de cas suspects</t>
-  </si>
-  <si>
-    <t>Nombre de municipalités qui ne signalent pas de cas suspects</t>
-  </si>
-  <si>
     <t>Trained team in the last 2 years</t>
   </si>
   <si>
@@ -7344,18 +7290,6 @@
     <t>Présence d'une équipe formée au cours des 2 dernières années (Score)</t>
   </si>
   <si>
-    <t>Porcentaje de municipios que no reportan casos sospechosos</t>
-  </si>
-  <si>
-    <t>Percentage of municipalities that do not report suspected cases</t>
-  </si>
-  <si>
-    <t>Proporção de municípios que não reportam casos suspeitos</t>
-  </si>
-  <si>
-    <t>Proportion de municipalités qui ne signalent pas de cas suspects</t>
-  </si>
-  <si>
     <t>Presencia de un equipo capacitado en los últimos 2 años</t>
   </si>
   <si>
@@ -7369,6 +7303,99 @@
   </si>
   <si>
     <t>Áreas subnacionais (estadual) com uma equipe que foi treinada para resposta a surtos nos últimos 2 anos</t>
+  </si>
+  <si>
+    <t>case_class_lab</t>
+  </si>
+  <si>
+    <t>Distribución espacial de municipios notificando casos de sarampión y rubeola</t>
+  </si>
+  <si>
+    <t>Número de municipios que reportan casos</t>
+  </si>
+  <si>
+    <t>case_class_infobox_text</t>
+  </si>
+  <si>
+    <t>case_class_legend_rep</t>
+  </si>
+  <si>
+    <t>case_class_legend_conf</t>
+  </si>
+  <si>
+    <t>Reporta casos confirmados</t>
+  </si>
+  <si>
+    <t>Número de municipios que reportan casos confirmados</t>
+  </si>
+  <si>
+    <t>case_class_lab_short</t>
+  </si>
+  <si>
+    <t>Casos reportados</t>
+  </si>
+  <si>
+    <t>Spatial distribution of municipalities reporting measles and rubella cases</t>
+  </si>
+  <si>
+    <t>Distribuição espacial dos municípios notificando casos de sarampo e rubéola</t>
+  </si>
+  <si>
+    <t>Distribution spatiale des municipalités signalant des cas de rougeole et de rubéole</t>
+  </si>
+  <si>
+    <t>Reports suspected cases</t>
+  </si>
+  <si>
+    <t>Reporta casos suspeitos</t>
+  </si>
+  <si>
+    <t>Number of municipalities reporting confirmed cases</t>
+  </si>
+  <si>
+    <t>Número de municípios que reportam casos confirmados</t>
+  </si>
+  <si>
+    <t>Nombre de municipalités signalant des cas confirmés</t>
+  </si>
+  <si>
+    <t>Reports confirmed cases</t>
+  </si>
+  <si>
+    <t>Signale des cas confirmés</t>
+  </si>
+  <si>
+    <t>Reported cases</t>
+  </si>
+  <si>
+    <t>Cas signalés</t>
+  </si>
+  <si>
+    <t>case_class_infobox_pct</t>
+  </si>
+  <si>
+    <t>Porcentaje de municipios que reportan casos confirmados</t>
+  </si>
+  <si>
+    <t>Percentage of municipalities reporting confirmed cases</t>
+  </si>
+  <si>
+    <t>Percentual de municípios que reportam casos confirmados</t>
+  </si>
+  <si>
+    <t>Pourcentage de municipalités signalant des cas confirmés</t>
+  </si>
+  <si>
+    <t>surv_table_cases_conf</t>
+  </si>
+  <si>
+    <t>Casos confirmados</t>
+  </si>
+  <si>
+    <t>Confirmed cases</t>
+  </si>
+  <si>
+    <t>Cas confirmés</t>
   </si>
 </sst>
 </file>
@@ -7927,7 +7954,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{064C7D9D-C4E2-B94C-B003-B8DCE10597B7}">
-  <dimension ref="A1:E174"/>
+  <dimension ref="A1:E176"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.83203125" bestFit="1" customWidth="1"/>
@@ -8938,21 +8965,21 @@
         <v>976</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" ht="31" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>1639</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>1631</v>
-      </c>
-      <c r="C60" s="15" t="s">
         <v>1632</v>
       </c>
+      <c r="B60" s="9" t="s">
+        <v>1651</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>1660</v>
+      </c>
       <c r="D60" s="3" t="s">
-        <v>1633</v>
+        <v>1661</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>1634</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
@@ -9232,16 +9259,16 @@
         <v>211</v>
       </c>
       <c r="B77" t="s">
-        <v>1644</v>
+        <v>1634</v>
       </c>
       <c r="C77" t="s">
-        <v>1655</v>
+        <v>1637</v>
       </c>
       <c r="D77" t="s">
-        <v>1671</v>
+        <v>1649</v>
       </c>
       <c r="E77" t="s">
-        <v>1661</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
@@ -10728,16 +10755,16 @@
         <v>421</v>
       </c>
       <c r="B165" t="s">
-        <v>1644</v>
+        <v>1634</v>
       </c>
       <c r="C165" t="s">
-        <v>1655</v>
+        <v>1637</v>
       </c>
       <c r="D165" t="s">
-        <v>1658</v>
+        <v>1640</v>
       </c>
       <c r="E165" t="s">
-        <v>1661</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.35">
@@ -10779,16 +10806,16 @@
         <v>425</v>
       </c>
       <c r="B168" t="s">
-        <v>1667</v>
+        <v>1645</v>
       </c>
       <c r="C168" t="s">
-        <v>1668</v>
+        <v>1646</v>
       </c>
       <c r="D168" t="s">
-        <v>1669</v>
+        <v>1647</v>
       </c>
       <c r="E168" t="s">
-        <v>1670</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.35">
@@ -10825,72 +10852,106 @@
         <v>1037</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" ht="31" x14ac:dyDescent="0.35">
       <c r="A171" s="7" t="s">
-        <v>1630</v>
+        <v>1650</v>
       </c>
       <c r="B171" s="9" t="s">
-        <v>1645</v>
-      </c>
-      <c r="C171" s="8" t="s">
-        <v>1648</v>
-      </c>
-      <c r="D171" s="7" t="s">
-        <v>1650</v>
-      </c>
-      <c r="E171" s="7" t="s">
-        <v>1652</v>
+        <v>1651</v>
+      </c>
+      <c r="C171" s="9" t="s">
+        <v>1660</v>
+      </c>
+      <c r="D171" s="3" t="s">
+        <v>1661</v>
+      </c>
+      <c r="E171" s="3" t="s">
+        <v>1662</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="7" t="s">
-        <v>1635</v>
+        <v>1654</v>
       </c>
       <c r="B172" s="9" t="s">
-        <v>1636</v>
-      </c>
-      <c r="C172" s="8" t="s">
-        <v>1642</v>
-      </c>
-      <c r="D172" s="7" t="s">
-        <v>1641</v>
-      </c>
-      <c r="E172" s="7" t="s">
-        <v>1637</v>
+        <v>1630</v>
+      </c>
+      <c r="C172" s="9" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D172" s="9" t="s">
+        <v>1664</v>
+      </c>
+      <c r="E172" s="9" t="s">
+        <v>1631</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="7" t="s">
-        <v>1638</v>
+        <v>1653</v>
       </c>
       <c r="B173" s="9" t="s">
-        <v>1646</v>
-      </c>
-      <c r="C173" s="7" t="s">
-        <v>1649</v>
-      </c>
-      <c r="D173" s="7" t="s">
-        <v>1651</v>
-      </c>
-      <c r="E173" s="7" t="s">
-        <v>1653</v>
+        <v>1657</v>
+      </c>
+      <c r="C173" s="9" t="s">
+        <v>1665</v>
+      </c>
+      <c r="D173" s="9" t="s">
+        <v>1666</v>
+      </c>
+      <c r="E173" s="9" t="s">
+        <v>1667</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="7" t="s">
-        <v>1640</v>
+        <v>1655</v>
       </c>
       <c r="B174" s="9" t="s">
-        <v>1663</v>
-      </c>
-      <c r="C174" s="7" t="s">
-        <v>1664</v>
-      </c>
-      <c r="D174" s="7" t="s">
-        <v>1665</v>
-      </c>
-      <c r="E174" s="7" t="s">
-        <v>1666</v>
+        <v>1656</v>
+      </c>
+      <c r="C174" s="9" t="s">
+        <v>1668</v>
+      </c>
+      <c r="D174" s="9" t="s">
+        <v>1656</v>
+      </c>
+      <c r="E174" s="9" t="s">
+        <v>1669</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A175" s="7" t="s">
+        <v>1658</v>
+      </c>
+      <c r="B175" s="9" t="s">
+        <v>1659</v>
+      </c>
+      <c r="C175" s="9" t="s">
+        <v>1670</v>
+      </c>
+      <c r="D175" s="9" t="s">
+        <v>1659</v>
+      </c>
+      <c r="E175" s="9" t="s">
+        <v>1671</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A176" s="7" t="s">
+        <v>1672</v>
+      </c>
+      <c r="B176" s="9" t="s">
+        <v>1673</v>
+      </c>
+      <c r="C176" s="9" t="s">
+        <v>1674</v>
+      </c>
+      <c r="D176" s="9" t="s">
+        <v>1675</v>
+      </c>
+      <c r="E176" s="9" t="s">
+        <v>1676</v>
       </c>
     </row>
   </sheetData>
@@ -12161,7 +12222,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01EA010-864B-8746-BF5D-2E469295667F}">
-  <dimension ref="A1:E198"/>
+  <dimension ref="A1:E201"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.5" bestFit="1" customWidth="1"/>
@@ -14109,738 +14170,738 @@
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>728</v>
+        <v>1677</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>729</v>
+        <v>1678</v>
       </c>
       <c r="C115" s="15" t="s">
-        <v>1245</v>
+        <v>1679</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>1585</v>
+        <v>1678</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>1433</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
+        <v>728</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>729</v>
+      </c>
+      <c r="C116" s="15" t="s">
+        <v>1245</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>1585</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>1433</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
         <v>730</v>
       </c>
-      <c r="B116" s="4" t="s">
+      <c r="B117" s="4" t="s">
         <v>731</v>
       </c>
-      <c r="C116" s="15" t="s">
+      <c r="C117" s="15" t="s">
         <v>1246</v>
       </c>
-      <c r="D116" s="3" t="s">
+      <c r="D117" s="3" t="s">
         <v>1586</v>
       </c>
-      <c r="E116" s="3" t="s">
+      <c r="E117" s="3" t="s">
         <v>1434</v>
       </c>
     </row>
-    <row r="117" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="A117" t="s">
+    <row r="118" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
         <v>732</v>
       </c>
-      <c r="B117" s="4" t="s">
+      <c r="B118" s="4" t="s">
         <v>733</v>
       </c>
-      <c r="C117" s="15" t="s">
+      <c r="C118" s="15" t="s">
         <v>1247</v>
       </c>
-      <c r="D117" s="3" t="s">
+      <c r="D118" s="3" t="s">
         <v>1587</v>
       </c>
-      <c r="E117" s="3" t="s">
+      <c r="E118" s="3" t="s">
         <v>1435</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A118" t="s">
-        <v>734</v>
-      </c>
-      <c r="B118" s="4" t="s">
-        <v>735</v>
-      </c>
-      <c r="C118" s="15" t="s">
-        <v>1248</v>
-      </c>
-      <c r="D118" s="3" t="s">
-        <v>1588</v>
-      </c>
-      <c r="E118" s="3" t="s">
-        <v>1436</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>737</v>
-      </c>
-      <c r="C119" s="13" t="s">
-        <v>738</v>
+        <v>735</v>
+      </c>
+      <c r="C119" s="15" t="s">
+        <v>1248</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>739</v>
+        <v>1588</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>1437</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>741</v>
-      </c>
-      <c r="C120" s="15" t="s">
-        <v>1249</v>
+        <v>737</v>
+      </c>
+      <c r="C120" s="13" t="s">
+        <v>738</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>1589</v>
+        <v>739</v>
       </c>
       <c r="E120" s="3" t="s">
-        <v>1438</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
+        <v>740</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>741</v>
+      </c>
+      <c r="C121" s="15" t="s">
+        <v>1249</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>1589</v>
+      </c>
+      <c r="E121" s="3" t="s">
+        <v>1438</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
         <v>742</v>
       </c>
-      <c r="B121" s="4" t="s">
+      <c r="B122" s="4" t="s">
         <v>743</v>
       </c>
-      <c r="C121" s="13" t="s">
+      <c r="C122" s="13" t="s">
         <v>1250</v>
       </c>
-      <c r="D121" s="3" t="s">
+      <c r="D122" s="3" t="s">
         <v>744</v>
       </c>
-      <c r="E121" s="3" t="s">
+      <c r="E122" s="3" t="s">
         <v>1439</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="A122" t="s">
-        <v>745</v>
-      </c>
-      <c r="B122" s="4" t="s">
-        <v>746</v>
-      </c>
-      <c r="C122" s="15" t="s">
-        <v>1251</v>
-      </c>
-      <c r="D122" s="3" t="s">
-        <v>1590</v>
-      </c>
-      <c r="E122" s="3" t="s">
-        <v>1440</v>
       </c>
     </row>
     <row r="123" spans="1:5" ht="31" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="C123" s="15" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>1591</v>
+        <v>1590</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>1441</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="124" spans="1:5" ht="31" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
+        <v>747</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>748</v>
+      </c>
+      <c r="C124" s="15" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>1591</v>
+      </c>
+      <c r="E124" s="3" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
         <v>749</v>
       </c>
-      <c r="B124" s="4" t="s">
+      <c r="B125" s="4" t="s">
         <v>750</v>
       </c>
-      <c r="C124" s="15" t="s">
+      <c r="C125" s="15" t="s">
         <v>1253</v>
       </c>
-      <c r="D124" s="3" t="s">
+      <c r="D125" s="3" t="s">
         <v>1592</v>
       </c>
-      <c r="E124" s="3" t="s">
+      <c r="E125" s="3" t="s">
         <v>1442</v>
-      </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A125" t="s">
-        <v>349</v>
-      </c>
-      <c r="B125" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="C125" s="15" t="s">
-        <v>916</v>
-      </c>
-      <c r="D125" s="3" t="s">
-        <v>1114</v>
-      </c>
-      <c r="E125" s="3" t="s">
-        <v>1021</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>1443</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="C127" s="13" t="s">
-        <v>355</v>
+        <v>352</v>
+      </c>
+      <c r="C127" s="15" t="s">
+        <v>917</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>356</v>
+        <v>1115</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>1444</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
+        <v>353</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="C128" s="13" t="s">
+        <v>355</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="E128" s="3" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
         <v>358</v>
       </c>
-      <c r="B128" s="4" t="s">
+      <c r="B129" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="C128" s="13" t="s">
+      <c r="C129" s="13" t="s">
         <v>360</v>
       </c>
-      <c r="D128" s="3" t="s">
+      <c r="D129" s="3" t="s">
         <v>361</v>
       </c>
-      <c r="E128" s="3" t="s">
+      <c r="E129" s="3" t="s">
         <v>1445</v>
       </c>
     </row>
-    <row r="129" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="A129" t="s">
+    <row r="130" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
         <v>363</v>
       </c>
-      <c r="B129" s="4" t="s">
+      <c r="B130" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C129" s="15" t="s">
+      <c r="C130" s="15" t="s">
         <v>876</v>
       </c>
-      <c r="D129" s="3" t="s">
+      <c r="D130" s="3" t="s">
         <v>1079</v>
       </c>
-      <c r="E129" s="3" t="s">
+      <c r="E130" s="3" t="s">
         <v>978</v>
-      </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A130" t="s">
-        <v>365</v>
-      </c>
-      <c r="B130" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C130" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="D130" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="E130" s="3" t="s">
-        <v>1446</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C131" s="13" t="s">
-        <v>1254</v>
+        <v>172</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C132" s="13" t="s">
-        <v>182</v>
+        <v>1254</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C133" s="13" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>370</v>
-      </c>
-      <c r="C134" s="15" t="s">
-        <v>918</v>
+        <v>186</v>
+      </c>
+      <c r="C134" s="13" t="s">
+        <v>187</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>1593</v>
+        <v>188</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>1024</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C135" s="15" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>1594</v>
+        <v>1593</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>751</v>
+        <v>371</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C136" s="13" t="s">
-        <v>172</v>
+        <v>372</v>
+      </c>
+      <c r="C136" s="15" t="s">
+        <v>919</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>173</v>
+        <v>1594</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>1446</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>753</v>
-      </c>
-      <c r="C137" s="15" t="s">
-        <v>1255</v>
+        <v>171</v>
+      </c>
+      <c r="C137" s="13" t="s">
+        <v>172</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>1595</v>
+        <v>173</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>1450</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="C138" s="13" t="s">
-        <v>1254</v>
+        <v>753</v>
+      </c>
+      <c r="C138" s="15" t="s">
+        <v>1255</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>178</v>
+        <v>1595</v>
       </c>
       <c r="E138" s="3" t="s">
-        <v>1447</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>756</v>
-      </c>
-      <c r="C139" s="15" t="s">
-        <v>1256</v>
+        <v>176</v>
+      </c>
+      <c r="C139" s="13" t="s">
+        <v>1254</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>1596</v>
+        <v>178</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>1451</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="C140" s="15" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>1597</v>
+        <v>1596</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>1452</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="C141" s="15" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>1598</v>
+        <v>1597</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>1453</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="C142" s="15" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>1599</v>
+        <v>1598</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>1454</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="C143" s="15" t="s">
-        <v>1169</v>
+        <v>1259</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>1600</v>
+        <v>1599</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>1455</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="C144" s="15" t="s">
-        <v>1260</v>
+        <v>1169</v>
       </c>
       <c r="D144" s="3" t="s">
-        <v>1601</v>
+        <v>1600</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>1456</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>373</v>
+        <v>765</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>374</v>
-      </c>
-      <c r="C145" s="13" t="s">
-        <v>375</v>
+        <v>766</v>
+      </c>
+      <c r="C145" s="15" t="s">
+        <v>1260</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>376</v>
+        <v>1601</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>1457</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>767</v>
+        <v>373</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>768</v>
-      </c>
-      <c r="C146" s="15" t="s">
-        <v>1261</v>
+        <v>374</v>
+      </c>
+      <c r="C146" s="13" t="s">
+        <v>375</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>1602</v>
+        <v>376</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="C147" s="13" t="s">
-        <v>304</v>
+        <v>768</v>
+      </c>
+      <c r="C147" s="15" t="s">
+        <v>1261</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>305</v>
+        <v>1602</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>1376</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>771</v>
-      </c>
-      <c r="C148" s="15" t="s">
-        <v>1262</v>
+        <v>303</v>
+      </c>
+      <c r="C148" s="13" t="s">
+        <v>304</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>1603</v>
+        <v>305</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>1459</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="C149" s="15" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>773</v>
+        <v>1603</v>
       </c>
       <c r="E149" s="3" t="s">
-        <v>1460</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="C150" s="15" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>1604</v>
+        <v>773</v>
       </c>
       <c r="E150" s="3" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="C151" s="15" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="E151" s="3" t="s">
-        <v>1462</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>392</v>
+        <v>777</v>
       </c>
       <c r="C152" s="15" t="s">
-        <v>926</v>
+        <v>1265</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>1122</v>
+        <v>1605</v>
       </c>
       <c r="E152" s="3" t="s">
-        <v>1032</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>780</v>
+        <v>392</v>
       </c>
       <c r="C153" s="15" t="s">
-        <v>1266</v>
+        <v>926</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>1606</v>
+        <v>1122</v>
       </c>
       <c r="E153" s="3" t="s">
-        <v>1463</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="C154" s="15" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="E154" s="3" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
+        <v>781</v>
+      </c>
+      <c r="B155" s="4" t="s">
+        <v>782</v>
+      </c>
+      <c r="C155" s="15" t="s">
+        <v>1267</v>
+      </c>
+      <c r="D155" s="3" t="s">
+        <v>1607</v>
+      </c>
+      <c r="E155" s="3" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
         <v>783</v>
       </c>
-      <c r="B155" s="4" t="s">
+      <c r="B156" s="4" t="s">
         <v>784</v>
       </c>
-      <c r="C155" s="15" t="s">
+      <c r="C156" s="15" t="s">
         <v>1268</v>
       </c>
-      <c r="D155" s="3" t="s">
+      <c r="D156" s="3" t="s">
         <v>1608</v>
       </c>
-      <c r="E155" s="3" t="s">
+      <c r="E156" s="3" t="s">
         <v>1465</v>
       </c>
     </row>
-    <row r="156" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="A156" t="s">
+    <row r="157" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
         <v>378</v>
       </c>
-      <c r="B156" s="4" t="s">
+      <c r="B157" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="C156" s="15" t="s">
+      <c r="C157" s="15" t="s">
         <v>920</v>
       </c>
-      <c r="D156" s="3" t="s">
+      <c r="D157" s="3" t="s">
         <v>1116</v>
       </c>
-      <c r="E156" s="3" t="s">
+      <c r="E157" s="3" t="s">
         <v>1026</v>
-      </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A157" t="s">
-        <v>380</v>
-      </c>
-      <c r="B157" s="4" t="s">
-        <v>374</v>
-      </c>
-      <c r="C157" s="13" t="s">
-        <v>375</v>
-      </c>
-      <c r="D157" s="3" t="s">
-        <v>376</v>
-      </c>
-      <c r="E157" s="3" t="s">
-        <v>1457</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>785</v>
+        <v>380</v>
       </c>
       <c r="B158" s="4" t="s">
         <v>374</v>
@@ -14857,686 +14918,737 @@
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>787</v>
-      </c>
-      <c r="C159" s="15" t="s">
-        <v>1269</v>
+        <v>374</v>
+      </c>
+      <c r="C159" s="13" t="s">
+        <v>375</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>1609</v>
+        <v>376</v>
       </c>
       <c r="E159" s="3" t="s">
-        <v>1466</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="C160" s="15" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="E160" s="3" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>381</v>
+        <v>788</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="C161" s="15" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="E161" s="3" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>384</v>
+        <v>790</v>
       </c>
       <c r="C162" s="15" t="s">
-        <v>922</v>
+        <v>1271</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>1118</v>
+        <v>1611</v>
       </c>
       <c r="E162" s="3" t="s">
-        <v>1028</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
+        <v>383</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="C163" s="15" t="s">
+        <v>922</v>
+      </c>
+      <c r="D163" s="3" t="s">
+        <v>1118</v>
+      </c>
+      <c r="E163" s="3" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A164" t="s">
         <v>385</v>
       </c>
-      <c r="B163" s="4" t="s">
+      <c r="B164" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="C163" s="15" t="s">
+      <c r="C164" s="15" t="s">
         <v>923</v>
       </c>
-      <c r="D163" s="3" t="s">
+      <c r="D164" s="3" t="s">
         <v>1119</v>
       </c>
-      <c r="E163" s="3" t="s">
+      <c r="E164" s="3" t="s">
         <v>1029</v>
       </c>
     </row>
-    <row r="164" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="A164" t="s">
+    <row r="165" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A165" t="s">
         <v>387</v>
       </c>
-      <c r="B164" s="4" t="s">
+      <c r="B165" s="4" t="s">
         <v>388</v>
       </c>
-      <c r="C164" s="15" t="s">
+      <c r="C165" s="15" t="s">
         <v>924</v>
       </c>
-      <c r="D164" s="3" t="s">
+      <c r="D165" s="3" t="s">
         <v>1120</v>
       </c>
-      <c r="E164" s="3" t="s">
+      <c r="E165" s="3" t="s">
         <v>1030</v>
-      </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A165" t="s">
-        <v>389</v>
-      </c>
-      <c r="B165" s="4" t="s">
-        <v>390</v>
-      </c>
-      <c r="C165" s="15" t="s">
-        <v>925</v>
-      </c>
-      <c r="D165" s="3" t="s">
-        <v>1121</v>
-      </c>
-      <c r="E165" s="3" t="s">
-        <v>1031</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C166" s="15" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="E166" s="3" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C167" s="15" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="E167" s="3" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C168" s="15" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="E168" s="3" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
+        <v>395</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="C169" s="15" t="s">
+        <v>928</v>
+      </c>
+      <c r="D169" s="3" t="s">
+        <v>1124</v>
+      </c>
+      <c r="E169" s="3" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A170" t="s">
         <v>397</v>
       </c>
-      <c r="B169" s="4" t="s">
+      <c r="B170" s="4" t="s">
         <v>398</v>
       </c>
-      <c r="C169" s="15" t="s">
+      <c r="C170" s="15" t="s">
         <v>929</v>
       </c>
-      <c r="D169" s="3" t="s">
+      <c r="D170" s="3" t="s">
         <v>1125</v>
       </c>
-      <c r="E169" s="3" t="s">
+      <c r="E170" s="3" t="s">
         <v>1035</v>
       </c>
     </row>
-    <row r="170" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A170" t="s">
+    <row r="171" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
+      <c r="A171" t="s">
         <v>791</v>
       </c>
-      <c r="B170" s="4" t="s">
+      <c r="B171" s="4" t="s">
         <v>792</v>
       </c>
-      <c r="C170" s="15" t="s">
+      <c r="C171" s="15" t="s">
         <v>1272</v>
       </c>
-      <c r="D170" s="3" t="s">
+      <c r="D171" s="3" t="s">
         <v>1612</v>
       </c>
-      <c r="E170" s="3" t="s">
+      <c r="E171" s="3" t="s">
         <v>1469</v>
       </c>
     </row>
-    <row r="171" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="A171" t="s">
+    <row r="172" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A172" t="s">
         <v>793</v>
       </c>
-      <c r="B171" s="4" t="s">
+      <c r="B172" s="4" t="s">
         <v>794</v>
       </c>
-      <c r="C171" s="15" t="s">
+      <c r="C172" s="15" t="s">
         <v>1273</v>
       </c>
-      <c r="D171" s="3" t="s">
+      <c r="D172" s="3" t="s">
         <v>1613</v>
       </c>
-      <c r="E171" s="3" t="s">
+      <c r="E172" s="3" t="s">
         <v>1470</v>
       </c>
     </row>
-    <row r="172" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A172" t="s">
+    <row r="173" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
+      <c r="A173" t="s">
         <v>795</v>
       </c>
-      <c r="B172" s="4" t="s">
+      <c r="B173" s="4" t="s">
         <v>796</v>
       </c>
-      <c r="C172" s="15" t="s">
+      <c r="C173" s="15" t="s">
         <v>1274</v>
       </c>
-      <c r="D172" s="3" t="s">
+      <c r="D173" s="3" t="s">
         <v>1614</v>
       </c>
-      <c r="E172" s="3" t="s">
+      <c r="E173" s="3" t="s">
         <v>1471</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A173" t="s">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A174" t="s">
         <v>797</v>
       </c>
-      <c r="B173" s="4" t="s">
+      <c r="B174" s="4" t="s">
         <v>390</v>
       </c>
-      <c r="C173" s="15" t="s">
+      <c r="C174" s="15" t="s">
         <v>925</v>
       </c>
-      <c r="D173" s="3" t="s">
+      <c r="D174" s="3" t="s">
         <v>1121</v>
       </c>
-      <c r="E173" s="3" t="s">
+      <c r="E174" s="3" t="s">
         <v>1472</v>
       </c>
     </row>
-    <row r="174" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="A174" t="s">
+    <row r="175" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A175" t="s">
         <v>798</v>
       </c>
-      <c r="B174" s="4" t="s">
+      <c r="B175" s="4" t="s">
         <v>799</v>
       </c>
-      <c r="C174" s="15" t="s">
+      <c r="C175" s="15" t="s">
         <v>1275</v>
       </c>
-      <c r="D174" s="3" t="s">
+      <c r="D175" s="3" t="s">
         <v>1615</v>
       </c>
-      <c r="E174" s="3" t="s">
+      <c r="E175" s="3" t="s">
         <v>1473</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A175" t="s">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A176" t="s">
         <v>800</v>
       </c>
-      <c r="B175" s="4" t="s">
+      <c r="B176" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="C175" s="15" t="s">
+      <c r="C176" s="15" t="s">
         <v>927</v>
       </c>
-      <c r="D175" s="3" t="s">
+      <c r="D176" s="3" t="s">
         <v>1123</v>
       </c>
-      <c r="E175" s="3" t="s">
+      <c r="E176" s="3" t="s">
         <v>1033</v>
-      </c>
-    </row>
-    <row r="176" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A176" t="s">
-        <v>801</v>
-      </c>
-      <c r="B176" s="4" t="s">
-        <v>802</v>
-      </c>
-      <c r="C176" s="15" t="s">
-        <v>1276</v>
-      </c>
-      <c r="D176" s="3" t="s">
-        <v>1616</v>
-      </c>
-      <c r="E176" s="3" t="s">
-        <v>1474</v>
       </c>
     </row>
     <row r="177" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
+        <v>801</v>
+      </c>
+      <c r="B177" s="4" t="s">
+        <v>802</v>
+      </c>
+      <c r="C177" s="15" t="s">
+        <v>1276</v>
+      </c>
+      <c r="D177" s="3" t="s">
+        <v>1616</v>
+      </c>
+      <c r="E177" s="3" t="s">
+        <v>1474</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
+      <c r="A178" t="s">
         <v>803</v>
       </c>
-      <c r="B177" s="4" t="s">
+      <c r="B178" s="4" t="s">
         <v>804</v>
       </c>
-      <c r="C177" s="15" t="s">
+      <c r="C178" s="15" t="s">
         <v>1277</v>
       </c>
-      <c r="D177" s="3" t="s">
+      <c r="D178" s="3" t="s">
         <v>1617</v>
       </c>
-      <c r="E177" s="3" t="s">
+      <c r="E178" s="3" t="s">
         <v>1475</v>
-      </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A178" t="s">
-        <v>399</v>
-      </c>
-      <c r="B178" s="4" t="s">
-        <v>400</v>
-      </c>
-      <c r="C178" s="15" t="s">
-        <v>930</v>
-      </c>
-      <c r="D178" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="E178" s="3" t="s">
-        <v>1036</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C179" s="15" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>1126</v>
+        <v>400</v>
       </c>
       <c r="E179" s="3" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="C180" s="13" t="s">
-        <v>405</v>
+        <v>402</v>
+      </c>
+      <c r="C180" s="15" t="s">
+        <v>931</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>406</v>
+        <v>1126</v>
       </c>
       <c r="E180" s="3" t="s">
-        <v>1476</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="C181" s="13" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="D181" s="3" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E181" s="3" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="C182" s="15" t="s">
-        <v>932</v>
+        <v>409</v>
+      </c>
+      <c r="C182" s="13" t="s">
+        <v>409</v>
       </c>
       <c r="D182" s="3" t="s">
-        <v>1127</v>
+        <v>410</v>
       </c>
       <c r="E182" s="3" t="s">
-        <v>1038</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="C183" s="13" t="s">
-        <v>1172</v>
+        <v>413</v>
+      </c>
+      <c r="C183" s="15" t="s">
+        <v>932</v>
       </c>
       <c r="D183" s="3" t="s">
-        <v>417</v>
+        <v>1127</v>
       </c>
       <c r="E183" s="3" t="s">
-        <v>1478</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="C184" s="15" t="s">
-        <v>933</v>
+        <v>415</v>
+      </c>
+      <c r="C184" s="13" t="s">
+        <v>1172</v>
       </c>
       <c r="D184" s="3" t="s">
-        <v>1128</v>
+        <v>417</v>
       </c>
       <c r="E184" s="3" t="s">
-        <v>1039</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
+        <v>419</v>
+      </c>
+      <c r="B185" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="C185" s="15" t="s">
+        <v>933</v>
+      </c>
+      <c r="D185" s="3" t="s">
+        <v>1128</v>
+      </c>
+      <c r="E185" s="3" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A186" t="s">
         <v>421</v>
       </c>
-      <c r="B185" s="4" t="s">
+      <c r="B186" s="4" t="s">
+        <v>1633</v>
+      </c>
+      <c r="C186" s="15" t="s">
+        <v>1636</v>
+      </c>
+      <c r="D186" t="s">
+        <v>1639</v>
+      </c>
+      <c r="E186" t="s">
+        <v>1642</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+      <c r="A187" t="s">
+        <v>805</v>
+      </c>
+      <c r="B187" s="20" t="s">
+        <v>1634</v>
+      </c>
+      <c r="C187" t="s">
+        <v>1637</v>
+      </c>
+      <c r="D187" t="s">
+        <v>1640</v>
+      </c>
+      <c r="E187" t="s">
         <v>1643</v>
-      </c>
-      <c r="C185" s="15" t="s">
-        <v>1654</v>
-      </c>
-      <c r="D185" t="s">
-        <v>1657</v>
-      </c>
-      <c r="E185" t="s">
-        <v>1660</v>
-      </c>
-    </row>
-    <row r="186" spans="1:5" ht="16" x14ac:dyDescent="0.4">
-      <c r="A186" t="s">
-        <v>805</v>
-      </c>
-      <c r="B186" s="20" t="s">
-        <v>1644</v>
-      </c>
-      <c r="C186" t="s">
-        <v>1655</v>
-      </c>
-      <c r="D186" t="s">
-        <v>1658</v>
-      </c>
-      <c r="E186" t="s">
-        <v>1661</v>
-      </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A187" t="s">
-        <v>422</v>
-      </c>
-      <c r="B187" s="4" t="s">
-        <v>423</v>
-      </c>
-      <c r="C187" s="15" t="s">
-        <v>934</v>
-      </c>
-      <c r="D187" s="3" t="s">
-        <v>1129</v>
-      </c>
-      <c r="E187" s="3" t="s">
-        <v>1040</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="C188" s="15" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="E188" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>1643</v>
+        <v>420</v>
       </c>
       <c r="C189" s="15" t="s">
-        <v>1654</v>
-      </c>
-      <c r="D189" t="s">
-        <v>1657</v>
-      </c>
-      <c r="E189" t="s">
-        <v>1660</v>
+        <v>933</v>
+      </c>
+      <c r="D189" s="3" t="s">
+        <v>1128</v>
+      </c>
+      <c r="E189" s="3" t="s">
+        <v>1039</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>400</v>
+        <v>1633</v>
       </c>
       <c r="C190" s="15" t="s">
-        <v>930</v>
-      </c>
-      <c r="D190" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="E190" s="3" t="s">
-        <v>1036</v>
+        <v>1636</v>
+      </c>
+      <c r="D190" t="s">
+        <v>1639</v>
+      </c>
+      <c r="E190" t="s">
+        <v>1642</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C191" s="15" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="D191" s="3" t="s">
-        <v>1126</v>
+        <v>400</v>
       </c>
       <c r="E191" s="3" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>806</v>
+        <v>427</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>420</v>
+        <v>402</v>
       </c>
       <c r="C192" s="15" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="D192" s="3" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="E192" s="3" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>808</v>
+        <v>420</v>
       </c>
       <c r="C193" s="15" t="s">
-        <v>1278</v>
+        <v>933</v>
       </c>
       <c r="D193" s="3" t="s">
-        <v>1618</v>
+        <v>1128</v>
       </c>
       <c r="E193" s="3" t="s">
-        <v>1479</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
+        <v>807</v>
+      </c>
+      <c r="B194" s="4" t="s">
+        <v>808</v>
+      </c>
+      <c r="C194" s="15" t="s">
+        <v>1278</v>
+      </c>
+      <c r="D194" s="3" t="s">
+        <v>1618</v>
+      </c>
+      <c r="E194" s="3" t="s">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A195" t="s">
         <v>809</v>
       </c>
-      <c r="B194" s="4" t="s">
-        <v>1643</v>
-      </c>
-      <c r="C194" s="15" t="s">
+      <c r="B195" s="4" t="s">
+        <v>1633</v>
+      </c>
+      <c r="C195" s="15" t="s">
+        <v>1636</v>
+      </c>
+      <c r="D195" t="s">
+        <v>1639</v>
+      </c>
+      <c r="E195" t="s">
+        <v>1642</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A196" t="s">
+        <v>810</v>
+      </c>
+      <c r="B196" s="4" t="s">
+        <v>1635</v>
+      </c>
+      <c r="C196" s="15" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D196" t="s">
+        <v>1641</v>
+      </c>
+      <c r="E196" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A197" s="7" t="s">
+        <v>1650</v>
+      </c>
+      <c r="B197" s="9" t="s">
+        <v>1651</v>
+      </c>
+      <c r="C197" s="9" t="s">
+        <v>1651</v>
+      </c>
+      <c r="D197" s="9" t="s">
+        <v>1651</v>
+      </c>
+      <c r="E197" s="9" t="s">
+        <v>1651</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A198" s="7" t="s">
         <v>1654</v>
       </c>
-      <c r="D194" t="s">
+      <c r="B198" s="9" t="s">
+        <v>1630</v>
+      </c>
+      <c r="C198" s="9" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D198" s="9" t="s">
+        <v>1630</v>
+      </c>
+      <c r="E198" s="9" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+      <c r="A199" s="7" t="s">
+        <v>1653</v>
+      </c>
+      <c r="B199" s="9" t="s">
         <v>1657</v>
       </c>
-      <c r="E194" t="s">
-        <v>1660</v>
-      </c>
-    </row>
-    <row r="195" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="A195" t="s">
-        <v>810</v>
-      </c>
-      <c r="B195" s="4" t="s">
-        <v>1647</v>
-      </c>
-      <c r="C195" s="15" t="s">
+      <c r="C199" s="9" t="s">
+        <v>1652</v>
+      </c>
+      <c r="D199" s="9" t="s">
+        <v>1652</v>
+      </c>
+      <c r="E199" s="9" t="s">
+        <v>1652</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A200" s="7" t="s">
+        <v>1655</v>
+      </c>
+      <c r="B200" s="9" t="s">
         <v>1656</v>
       </c>
-      <c r="D195" t="s">
+      <c r="C200" s="9" t="s">
+        <v>1656</v>
+      </c>
+      <c r="D200" s="9" t="s">
+        <v>1656</v>
+      </c>
+      <c r="E200" s="9" t="s">
+        <v>1656</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A201" s="7" t="s">
+        <v>1658</v>
+      </c>
+      <c r="B201" s="9" t="s">
         <v>1659</v>
       </c>
-      <c r="E195" t="s">
-        <v>1662</v>
-      </c>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A196" s="7" t="s">
-        <v>1630</v>
-      </c>
-      <c r="B196" s="9" t="s">
-        <v>1645</v>
-      </c>
-      <c r="C196" s="8" t="s">
-        <v>1648</v>
-      </c>
-      <c r="D196" s="7" t="s">
-        <v>1650</v>
-      </c>
-      <c r="E196" s="7" t="s">
-        <v>1652</v>
-      </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A197" s="7" t="s">
-        <v>1635</v>
-      </c>
-      <c r="B197" s="9" t="s">
-        <v>1636</v>
-      </c>
-      <c r="C197" s="8" t="s">
-        <v>1642</v>
-      </c>
-      <c r="D197" s="7" t="s">
-        <v>1641</v>
-      </c>
-      <c r="E197" s="7" t="s">
-        <v>1637</v>
-      </c>
-    </row>
-    <row r="198" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="A198" s="7" t="s">
-        <v>1638</v>
-      </c>
-      <c r="B198" s="9" t="s">
-        <v>1646</v>
-      </c>
-      <c r="C198" s="7" t="s">
-        <v>1649</v>
-      </c>
-      <c r="D198" s="7" t="s">
-        <v>1651</v>
-      </c>
-      <c r="E198" s="7" t="s">
-        <v>1653</v>
+      <c r="C201" s="9" t="s">
+        <v>1659</v>
+      </c>
+      <c r="D201" s="9" t="s">
+        <v>1659</v>
+      </c>
+      <c r="E201" s="9" t="s">
+        <v>1659</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E195" xr:uid="{B01EA010-864B-8746-BF5D-2E469295667F}"/>
+  <autoFilter ref="A1:E196" xr:uid="{B01EA010-864B-8746-BF5D-2E469295667F}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Added all corrections to dashboard and reports
</commit_message>
<xml_diff>
--- a/src/R/translations.xlsx
+++ b/src/R/translations.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2921" uniqueCount="2921">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3075" uniqueCount="3075">
   <si>
     <t>LABEL</t>
   </si>
@@ -8779,6 +8779,468 @@
   </si>
   <si>
     <t xml:space="preserve">Génération du rapport, veuillez patienter...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acerca de</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sobre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À propos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lorem ipsum dolor sit amet, consectetur adipiscing elit. Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_what_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Qué es?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is it?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O que é?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qu'est-ce que c'est ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_what_body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La sostenibilidad de la eliminación de la poliomielitis, el sarampión y la rubéola en la Región de las Américas requiere un monitoreo continuo del riesgo para orientar acciones de mitigación oportunas y efectivas. Esta sección presenta la visualización conjunta del análisis de riesgo de polio y el de sarampión y rubéola, utilizando el puntaje total y los componentes compartidos de inmunidad poblacional y calidad de la vigilancia. La visualización conjunta del riesgo no genera un puntaje numérico, sino una clasificación cualitativa del riesgo. Los puntajes individuales de cada análisis se presentan como referencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sustaining the elimination of poliomyelitis, measles, and rubella in the Region of the Americas requires continuous risk monitoring to guide timely and effective mitigation actions. This section presents the joint visualization of the polio risk analysis and the measles and rubella risk analysis, using the total score and the shared components of population immunity and surveillance quality. The joint risk visualization does not generate a numerical score, but rather a qualitative risk classification. The individual scores from each analysis are presented as a reference.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A sustentabilidade da eliminação da poliomielite, do sarampo e da rubéola na Região das Américas requer monitoramento contínuo do risco para orientar ações de mitigação oportunas e eficazes. Esta seção apresenta a visualização conjunta da análise de risco de poliomielite e da análise de risco de sarampo e rubéola, utilizando a pontuação total e os componentes compartilhados de imunidade populacional e qualidade da vigilância. A visualização conjunta do risco não gera uma pontuação numérica, mas sim uma classificação qualitativa do risco. As pontuações individuais de cada análise são apresentadas como referência.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pérennisation de l'élimination de la poliomyélite, de la rougeole et de la rubéole dans la Région des Amériques nécessite une surveillance continue du risque afin d'orienter des actions d'atténuation rapides et efficaces. Cette section présente la visualisation conjointe de l'analyse du risque de poliomyélite et de celle du risque de rougeole et de rubéole, en utilisant le score total et les composantes partagées d'immunité de la population et de qualité de la surveillance. La visualisation conjointe du risque ne génère pas de score numérique, mais plutôt une classification qualitative du risque. Les scores individuels de chaque analyse sont présentés à titre de référence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_scale_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Cuál es la escala de puntaje por análisis?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the scoring scale for each analysis?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qual é a escala de pontuação por análise?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quelle est l'échelle de score par analyse ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_scale_intro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las variables y la categorización del riesgo difieren entre ambos análisis. En la tabla 1, se presentan las categorías de riesgo y las puntuaciones respectivas para cada análisis:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The variables and risk categorization differ between the two analyses. Table 1 presents the risk categories and corresponding scores for each analysis:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As variáveis e a categorização do risco diferem entre as duas análises. Na tabela 1, são apresentadas as categorias de risco e as respectivas pontuações para cada análise:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les variables et la catégorisation du risque diffèrent entre les deux analyses. Le tableau 1 présente les catégories de risque et les scores respectifs pour chaque analyse :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_scale_table_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabla 1: Puntaje de riesgo asignado a nivel de municipio para polio, sarampión y rubeola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table 1: Risk score assigned at municipality level for polio, measles, and rubella</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabela 1: Pontuação de risco atribuída em nível municipal para poliomielite, sarampo e rubéola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau 1 : Score de risque attribué au niveau municipal pour la poliomyélite, la rougeole et la rubéole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_scale_note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La categorización del riesgo para cada uno de los componentes del análisis de sarampión y rubeola se encuentra aquí. Para polio se encuentra aquí.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The risk categorization for each component of the measles and rubella analysis can be found here. For polio, it can be found here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A categorização do risco para cada um dos componentes da análise de sarampo e rubéola encontra-se aqui. Para poliomielite, encontra-se aqui.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La catégorisation du risque pour chacune des composantes de l'analyse de la rougeole et de la rubéole se trouve ici. Pour la poliomyélite, elle se trouve ici.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_matrix_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como se determina o risco conjunto?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_matrix_intro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se considera la categoría de mayor riesgo entre ambos análisis (ver tabla 2). Por ejemplo, si para el municipio X, el análisis de riesgo para polio fue “Alto”, y para sarampión y rubeola “Muy alto”, entonces la clasificación final de dicho municipio será “Muy alto”. Esta categorización se utiliza para el perfil de riesgo general derivado del puntaje total, así como para los componentes de inmunidad poblacional y calidad de la vigilancia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The higher-risk category between both analyses is used (see table 2). For example, if for municipality X, the polio risk analysis was “High” and the measles and rubella analysis was “Very high,” then the final classification for that municipality will be “Very high.” This categorization is used for the general risk profile derived from the total score, as well as for the population immunity and surveillance quality components.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Considera-se a categoria de maior risco entre as duas análises (ver tabela 2). Por exemplo, se para o município X, a análise de risco de poliomielite foi “Alto” e a de sarampo e rubéola foi “Muito alto”, então a classificação final desse município será “Muito alto”. Essa categorização é utilizada para o perfil de risco geral derivado da pontuação total, bem como para os componentes de imunidade populacional e qualidade da vigilância.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La catégorie de risque la plus élevée entre les deux analyses est retenue (voir tableau 2). Par exemple, si pour la municipalité X, l'analyse du risque de poliomyélite était « Élevé » et celle de la rougeole et de la rubéole « Très élevé », alors la classification finale de cette municipalité sera « Très élevé ». Cette catégorisation est utilisée pour le profil de risque général dérivé du score total, ainsi que pour les composantes d'immunité de la population et de qualité de la surveillance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_matrix_table_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabla 2: Visualización conjunta de los resultados del análisis de riesgo polio, sarampión y rubeola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table 2: Joint visualization of the polio, measles, and rubella risk analysis results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabela 2: Visualização conjunta dos resultados da análise de risco de poliomielite, sarampo e rubéola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau 2 : Visualisation conjointe des résultats de l'analyse du risque de poliomyélite, de rougeole et de rubéole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_matrix_note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los puntajes numéricos por cada enfermedad no son directamente comparables; sin embargo, las categorías de riesgo permiten una interpretación conjunta de los resultados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The numerical scores for each disease are not directly comparable; however, the risk categories allow for a joint interpretation of the results.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As pontuações numéricas de cada doença não são diretamente comparáveis; no entanto, as categorias de risco permitem uma interpretação conjunta dos resultados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les scores numériques de chaque maladie ne sont pas directement comparables ; cependant, les catégories de risque permettent une interprétation conjointe des résultats.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_order_note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La herramienta mostrará los puntajes individuales obtenidos para sarampión, rubeola y polio, por cada municipio. El orden por defecto que mostrará la herramienta será la suma de los puntajes obtenidos para sarampión, rubeola y polio. Sin embargo, la herramienta permitirá ordenar la relación de municipios, de mayor a menor, ya sea por los puntajes obtenidos por sarampión/rubeola o por polio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The tool will show the individual scores obtained for measles, rubella, and polio for each municipality. The tool's default order will be the sum of the scores obtained for measles, rubella, and polio. However, the tool will allow the list of municipalities to be sorted, from highest to lowest, by either the measles/rubella scores or the polio scores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A ferramenta mostrará as pontuações individuais obtidas para sarampo, rubéola e poliomielite, por município. A ordem padrão exibida pela ferramenta será a soma das pontuações obtidas para sarampo, rubéola e poliomielite. No entanto, a ferramenta permitirá ordenar a lista de municípios, do maior para o menor, seja pelas pontuações obtidas para sarampo/rubéola ou para poliomielite.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'outil affichera les scores individuels obtenus pour la rougeole, la rubéole et la poliomyélite, pour chaque municipalité. L'ordre par défaut affiché par l'outil sera la somme des scores obtenus pour la rougeole, la rubéole et la poliomyélite. Toutefois, l'outil permettra de trier la liste des municipalités, du plus élevé au plus faible, selon les scores obtenus pour la rougeole/rubéole ou pour la poliomyélite.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_results_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Cómo se obtienen los resultados?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How are the results obtained?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como são obtidos os resultados?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment les résultats sont-ils obtenus ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_results_body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se debe realizar el análisis de riesgo para poliomielitis, sarampión y rubéola. A partir de los resultados obtenidos, la herramienta permite integrar y visualizar de manera conjunta y automatizada dichos análisis, presentándolos en un tablero interactivo y en reportes generados en formatos HTML y Word.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The risk analysis for poliomyelitis, measles, and rubella must be carried out. Based on the results obtained, the tool integrates and visualizes these analyses jointly and automatically, presenting them in an interactive dashboard and in reports generated in HTML and Word formats.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deve-se realizar a análise de risco para poliomielite, sarampo e rubéola. A partir dos resultados obtidos, a ferramenta permite integrar e visualizar de forma conjunta e automatizada essas análises, apresentando-as em um painel interativo e em relatórios gerados nos formatos HTML e Word.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'analyse du risque de poliomyélite, de rougeole et de rubéole doit être réalisée. À partir des résultats obtenus, l'outil permet d'intégrer et de visualiser conjointement et automatiquement ces analyses, en les présentant dans un tableau de bord interactif et dans des rapports générés aux formats HTML et Word.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La categorización del riesgo para cada uno de los componentes del análisis de sarampión y rubeola se encuentra %s. Para polio se encuentra %s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The risk categorization for each component of the measles and rubella analysis can be found %s. For polio, it can be found %s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A categorização do risco para cada um dos componentes da análise de sarampo e rubéola encontra-se %s. Para poliomielite, encontra-se %s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La catégorisation du risque pour chacune des composantes de l'analyse de la rougeole et de la rubéole se trouve %s. Pour la poliomyélite, elle se trouve %s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_about_link_word</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aquí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">here</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aqui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ici</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visualización conjunta del riesgo de Polio, Sarampión y Rubéola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joint Visualization of Polio, Measles, and Rubella Risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visualização conjunta do risco de poliomielite, sarampo e rubéola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visualisation conjointe du risque de poliomyélite, de rougeole et de rubéole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_synthesis_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Síntesis comparativa de la distribución del riesgo por componente para polio, sarampión y rubeola. %s, %s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparative synthesis of risk distribution by component for polio, measles, and rubella. %s, %s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Síntese comparativa da distribuição do risco por componente para poliomielite, sarampo e rubéola. %s, %s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Synthèse comparative de la distribution du risque par composante pour la poliomyélite, la rougeole et la rubéole. %s, %s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_synthesis_col_component</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_synthesis_col_low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bajo riesgo (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low risk (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baixo risco (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risque faible (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_synthesis_col_medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riesgo medio (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium risk (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risco médio (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risque moyen (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_synthesis_col_high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alto riesgo (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High risk (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alto risco (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risque élevé (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_synthesis_col_very_high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muy alto riesgo (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very high risk (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risco muito alto (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risque très élevé (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_synthesis_row_general</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profil de risque général</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultados del riesgo conjunto por municipio para polio, sarampión y rubeola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joint risk results by municipality for polio, measles, and rubella</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultados do risco conjunto por município para poliomielite, sarampo e rubéola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultats du risque conjoint par municipalité pour la poliomyélite, la rougeole et la rubéole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mapa de clasificación de riesgo para polio, sarampión y rubéola por municipio - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk classification map for polio, measles, and rubella by municipality - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mapa de classificação de risco para poliomielite, sarampo e rubéola por município - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carte de classification du risque pour la poliomyélite, la rougeole et la rubéole par municipalité - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribución de municipios para polio, sarampión y rubeola según categoría de riesgo - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribution of municipalities for polio, measles, and rubella by risk category - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribuição de municípios para poliomielite, sarampo e rubéola segundo categoria de risco - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répartition des municipalités pour la poliomyélite, la rougeole et la rubéole selon la catégorie de risque - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_immunity_map_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribución espacial por categoría de riesgo e inmunidad poblacional para polio, sarampión y rubeola - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spatial distribution by risk category and population immunity for polio, measles, and rubella - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribuição espacial por categoria de risco e imunidade populacional para poliomielite, sarampo e rubéola - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répartition spatiale par catégorie de risque et immunité de la population pour la poliomyélite, la rougeole et la rubéole - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_immunity_distribution_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribución de municipios para polio, sarampión y rubeola según categoría de riesgo e inmunidad poblacional - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribution of municipalities for polio, measles, and rubella by risk category and population immunity - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribuição de municípios para poliomielite, sarampo e rubéola segundo categoria de risco e imunidade populacional - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répartition des municipalités pour la poliomyélite, la rougeole et la rubéole selon la catégorie de risque et l'immunité de la population - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_immunity_table_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultados del riesgo conjunto de inmunidad poblacional por municipio para polio, sarampión y rubeola - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joint population immunity risk results by municipality for polio, measles, and rubella - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultados do risco conjunto de imunidade populacional por município para poliomielite, sarampo e rubéola - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultats du risque conjoint d'immunité de la population par municipalité pour la poliomyélite, la rougeole et la rubéole - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_surveillance_map_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribución espacial por categoría de riesgo y calidad de la vigilancia para polio, sarampión y rubeola - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spatial distribution by risk category and surveillance quality for polio, measles, and rubella - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribuição espacial por categoria de risco e qualidade da vigilância para poliomielite, sarampo e rubéola - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répartition spatiale par catégorie de risque et qualité de la surveillance pour la poliomyélite, la rougeole et la rubéole - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_surveillance_distribution_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribución de municipios para polio, sarampión y rubeola según categoría de riesgo y calidad de la vigilancia - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribution of municipalities for polio, measles, and rubella by risk category and surveillance quality - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribuição de municípios para poliomielite, sarampo e rubéola segundo categoria de risco e qualidade da vigilância - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répartition des municipalités pour la poliomyélite, la rougeole et la rubéole selon la catégorie de risque et la qualité de la surveillance - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_surveillance_table_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultados del riesgo conjunto de calidad de la vigilancia por municipio para polio, sarampión y rubeola - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joint surveillance quality risk results by municipality for polio, measles, and rubella - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultados do risco conjunto de qualidade da vigilância por município para poliomielite, sarampo e rubéola - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultats du risque conjoint de qualité de la surveillance par municipalité pour la poliomyélite, la rougeole et la rubéole - %s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joint_barplot_xaxis_title</t>
   </si>
 </sst>
 </file>
@@ -16827,16 +17289,16 @@
         <v>2631</v>
       </c>
       <c r="B203" t="s">
-        <v>2632</v>
+        <v>2999</v>
       </c>
       <c r="C203" t="s">
-        <v>2633</v>
+        <v>3000</v>
       </c>
       <c r="D203" t="s">
-        <v>2634</v>
+        <v>3001</v>
       </c>
       <c r="E203" t="s">
-        <v>2635</v>
+        <v>3002</v>
       </c>
     </row>
     <row r="204">
@@ -16844,16 +17306,16 @@
         <v>2636</v>
       </c>
       <c r="B204" t="s">
-        <v>2637</v>
+        <v>3032</v>
       </c>
       <c r="C204" t="s">
-        <v>2638</v>
+        <v>3033</v>
       </c>
       <c r="D204" t="s">
-        <v>2639</v>
+        <v>3034</v>
       </c>
       <c r="E204" t="s">
-        <v>2640</v>
+        <v>3035</v>
       </c>
     </row>
     <row r="205">
@@ -16912,16 +17374,16 @@
         <v>2655</v>
       </c>
       <c r="B208" t="s">
-        <v>2656</v>
+        <v>3036</v>
       </c>
       <c r="C208" t="s">
-        <v>2657</v>
+        <v>3037</v>
       </c>
       <c r="D208" t="s">
-        <v>2658</v>
+        <v>3038</v>
       </c>
       <c r="E208" t="s">
-        <v>2659</v>
+        <v>3039</v>
       </c>
     </row>
     <row r="209">
@@ -16929,16 +17391,16 @@
         <v>2660</v>
       </c>
       <c r="B209" t="s">
-        <v>2661</v>
+        <v>3040</v>
       </c>
       <c r="C209" t="s">
-        <v>2662</v>
+        <v>3041</v>
       </c>
       <c r="D209" t="s">
-        <v>2663</v>
+        <v>3042</v>
       </c>
       <c r="E209" t="s">
-        <v>2664</v>
+        <v>3043</v>
       </c>
     </row>
     <row r="210">
@@ -17065,16 +17527,16 @@
         <v>2696</v>
       </c>
       <c r="B217" t="s">
-        <v>2697</v>
+        <v>2034</v>
       </c>
       <c r="C217" t="s">
-        <v>2698</v>
+        <v>2035</v>
       </c>
       <c r="D217" t="s">
-        <v>2699</v>
+        <v>2036</v>
       </c>
       <c r="E217" t="s">
-        <v>2700</v>
+        <v>2037</v>
       </c>
     </row>
     <row r="218">
@@ -17198,733 +17660,1158 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>2729</v>
+        <v>2748</v>
       </c>
       <c r="B225" t="s">
-        <v>2730</v>
+        <v>2749</v>
       </c>
       <c r="C225" t="s">
-        <v>2731</v>
+        <v>2750</v>
       </c>
       <c r="D225" t="s">
-        <v>2730</v>
+        <v>2751</v>
       </c>
       <c r="E225" t="s">
-        <v>2732</v>
+        <v>2752</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>2733</v>
+        <v>2753</v>
       </c>
       <c r="B226" t="s">
-        <v>2734</v>
+        <v>2754</v>
       </c>
       <c r="C226" t="s">
-        <v>2735</v>
+        <v>2755</v>
       </c>
       <c r="D226" t="s">
-        <v>2736</v>
+        <v>2756</v>
       </c>
       <c r="E226" t="s">
-        <v>2737</v>
+        <v>2757</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>2738</v>
+        <v>2758</v>
       </c>
       <c r="B227" t="s">
-        <v>2739</v>
+        <v>2759</v>
       </c>
       <c r="C227" t="s">
-        <v>2740</v>
+        <v>2760</v>
       </c>
       <c r="D227" t="s">
-        <v>2741</v>
+        <v>2761</v>
       </c>
       <c r="E227" t="s">
-        <v>2742</v>
+        <v>2762</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>2743</v>
+        <v>2763</v>
       </c>
       <c r="B228" t="s">
-        <v>2744</v>
+        <v>2764</v>
       </c>
       <c r="C228" t="s">
-        <v>2745</v>
+        <v>2765</v>
       </c>
       <c r="D228" t="s">
-        <v>2746</v>
+        <v>2766</v>
       </c>
       <c r="E228" t="s">
-        <v>2747</v>
+        <v>2767</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>2748</v>
+        <v>2768</v>
       </c>
       <c r="B229" t="s">
-        <v>2749</v>
+        <v>2769</v>
       </c>
       <c r="C229" t="s">
-        <v>2750</v>
+        <v>2770</v>
       </c>
       <c r="D229" t="s">
-        <v>2751</v>
+        <v>2771</v>
       </c>
       <c r="E229" t="s">
-        <v>2752</v>
+        <v>2772</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>2753</v>
+        <v>2773</v>
       </c>
       <c r="B230" t="s">
-        <v>2754</v>
+        <v>2774</v>
       </c>
       <c r="C230" t="s">
-        <v>2755</v>
+        <v>2775</v>
       </c>
       <c r="D230" t="s">
-        <v>2756</v>
+        <v>2776</v>
       </c>
       <c r="E230" t="s">
-        <v>2757</v>
+        <v>2777</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>2758</v>
+        <v>2778</v>
       </c>
       <c r="B231" t="s">
-        <v>2759</v>
+        <v>2779</v>
       </c>
       <c r="C231" t="s">
-        <v>2760</v>
+        <v>2780</v>
       </c>
       <c r="D231" t="s">
-        <v>2761</v>
+        <v>2781</v>
       </c>
       <c r="E231" t="s">
-        <v>2762</v>
+        <v>2782</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>2763</v>
+        <v>2783</v>
       </c>
       <c r="B232" t="s">
-        <v>2764</v>
+        <v>2784</v>
       </c>
       <c r="C232" t="s">
-        <v>2765</v>
+        <v>2785</v>
       </c>
       <c r="D232" t="s">
-        <v>2766</v>
+        <v>2786</v>
       </c>
       <c r="E232" t="s">
-        <v>2767</v>
+        <v>2787</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>2768</v>
+        <v>2788</v>
       </c>
       <c r="B233" t="s">
-        <v>2769</v>
+        <v>2789</v>
       </c>
       <c r="C233" t="s">
-        <v>2770</v>
+        <v>2790</v>
       </c>
       <c r="D233" t="s">
-        <v>2771</v>
+        <v>2791</v>
       </c>
       <c r="E233" t="s">
-        <v>2772</v>
+        <v>2792</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>2773</v>
+        <v>2793</v>
       </c>
       <c r="B234" t="s">
-        <v>2774</v>
+        <v>2794</v>
       </c>
       <c r="C234" t="s">
-        <v>2775</v>
+        <v>2795</v>
       </c>
       <c r="D234" t="s">
-        <v>2776</v>
+        <v>2796</v>
       </c>
       <c r="E234" t="s">
-        <v>2777</v>
+        <v>2797</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>2778</v>
+        <v>2798</v>
       </c>
       <c r="B235" t="s">
-        <v>2779</v>
+        <v>2799</v>
       </c>
       <c r="C235" t="s">
-        <v>2780</v>
+        <v>2800</v>
       </c>
       <c r="D235" t="s">
-        <v>2781</v>
+        <v>2801</v>
       </c>
       <c r="E235" t="s">
-        <v>2782</v>
+        <v>2802</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>2783</v>
+        <v>2803</v>
       </c>
       <c r="B236" t="s">
-        <v>2784</v>
+        <v>2804</v>
       </c>
       <c r="C236" t="s">
-        <v>2785</v>
+        <v>2805</v>
       </c>
       <c r="D236" t="s">
-        <v>2786</v>
+        <v>2806</v>
       </c>
       <c r="E236" t="s">
-        <v>2787</v>
+        <v>2805</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>2788</v>
+        <v>2807</v>
       </c>
       <c r="B237" t="s">
-        <v>2789</v>
+        <v>2808</v>
       </c>
       <c r="C237" t="s">
-        <v>2790</v>
+        <v>2809</v>
       </c>
       <c r="D237" t="s">
-        <v>2791</v>
+        <v>2810</v>
       </c>
       <c r="E237" t="s">
-        <v>2792</v>
+        <v>2811</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>2793</v>
+        <v>2812</v>
       </c>
       <c r="B238" t="s">
-        <v>2794</v>
+        <v>2813</v>
       </c>
       <c r="C238" t="s">
-        <v>2795</v>
+        <v>2814</v>
       </c>
       <c r="D238" t="s">
-        <v>2796</v>
+        <v>2815</v>
       </c>
       <c r="E238" t="s">
-        <v>2797</v>
+        <v>2816</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>2798</v>
+        <v>2817</v>
       </c>
       <c r="B239" t="s">
-        <v>2799</v>
+        <v>2818</v>
       </c>
       <c r="C239" t="s">
-        <v>2800</v>
+        <v>2819</v>
       </c>
       <c r="D239" t="s">
-        <v>2801</v>
+        <v>2820</v>
       </c>
       <c r="E239" t="s">
-        <v>2802</v>
+        <v>2821</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>2803</v>
+        <v>2822</v>
       </c>
       <c r="B240" t="s">
-        <v>2804</v>
+        <v>2185</v>
       </c>
       <c r="C240" t="s">
-        <v>2805</v>
+        <v>2186</v>
       </c>
       <c r="D240" t="s">
-        <v>2806</v>
+        <v>2185</v>
       </c>
       <c r="E240" t="s">
-        <v>2805</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>2807</v>
+        <v>2823</v>
       </c>
       <c r="B241" t="s">
-        <v>2808</v>
+        <v>1903</v>
       </c>
       <c r="C241" t="s">
-        <v>2809</v>
+        <v>1904</v>
       </c>
       <c r="D241" t="s">
-        <v>2810</v>
+        <v>1905</v>
       </c>
       <c r="E241" t="s">
-        <v>2811</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>2812</v>
+        <v>2824</v>
       </c>
       <c r="B242" t="s">
-        <v>2813</v>
+        <v>2825</v>
       </c>
       <c r="C242" t="s">
-        <v>2814</v>
+        <v>2826</v>
       </c>
       <c r="D242" t="s">
-        <v>2815</v>
+        <v>2827</v>
       </c>
       <c r="E242" t="s">
-        <v>2816</v>
+        <v>2828</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>2817</v>
+        <v>2829</v>
       </c>
       <c r="B243" t="s">
-        <v>2818</v>
+        <v>2830</v>
       </c>
       <c r="C243" t="s">
-        <v>2819</v>
+        <v>2831</v>
       </c>
       <c r="D243" t="s">
-        <v>2820</v>
+        <v>2832</v>
       </c>
       <c r="E243" t="s">
-        <v>2821</v>
+        <v>2833</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>2822</v>
+        <v>2834</v>
       </c>
       <c r="B244" t="s">
-        <v>2185</v>
+        <v>2858</v>
       </c>
       <c r="C244" t="s">
-        <v>2186</v>
+        <v>2859</v>
       </c>
       <c r="D244" t="s">
-        <v>2185</v>
+        <v>2860</v>
       </c>
       <c r="E244" t="s">
-        <v>2187</v>
+        <v>2861</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>2823</v>
+        <v>2839</v>
       </c>
       <c r="B245" t="s">
-        <v>1903</v>
+        <v>1952</v>
       </c>
       <c r="C245" t="s">
-        <v>1904</v>
+        <v>1953</v>
       </c>
       <c r="D245" t="s">
-        <v>1905</v>
+        <v>1954</v>
       </c>
       <c r="E245" t="s">
-        <v>1906</v>
+        <v>2840</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>2824</v>
+        <v>2841</v>
       </c>
       <c r="B246" t="s">
-        <v>2825</v>
+        <v>2842</v>
       </c>
       <c r="C246" t="s">
-        <v>2826</v>
+        <v>1958</v>
       </c>
       <c r="D246" t="s">
-        <v>2827</v>
+        <v>1959</v>
       </c>
       <c r="E246" t="s">
-        <v>2828</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>2829</v>
+        <v>2843</v>
       </c>
       <c r="B247" t="s">
-        <v>2830</v>
+        <v>1962</v>
       </c>
       <c r="C247" t="s">
-        <v>2831</v>
+        <v>1963</v>
       </c>
       <c r="D247" t="s">
-        <v>2832</v>
+        <v>1964</v>
       </c>
       <c r="E247" t="s">
-        <v>2833</v>
+        <v>1965</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>2834</v>
+        <v>2844</v>
       </c>
       <c r="B248" t="s">
-        <v>2858</v>
+        <v>2845</v>
       </c>
       <c r="C248" t="s">
-        <v>2859</v>
+        <v>1968</v>
       </c>
       <c r="D248" t="s">
-        <v>2860</v>
+        <v>1969</v>
       </c>
       <c r="E248" t="s">
-        <v>2861</v>
+        <v>1970</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>2839</v>
+        <v>2846</v>
       </c>
       <c r="B249" t="s">
-        <v>1952</v>
+        <v>2847</v>
       </c>
       <c r="C249" t="s">
-        <v>1953</v>
+        <v>2847</v>
       </c>
       <c r="D249" t="s">
-        <v>1954</v>
+        <v>2847</v>
       </c>
       <c r="E249" t="s">
-        <v>2840</v>
+        <v>2847</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>2841</v>
+        <v>2848</v>
       </c>
       <c r="B250" t="s">
-        <v>2842</v>
+        <v>2849</v>
       </c>
       <c r="C250" t="s">
-        <v>1958</v>
+        <v>2850</v>
       </c>
       <c r="D250" t="s">
-        <v>1959</v>
+        <v>2851</v>
       </c>
       <c r="E250" t="s">
-        <v>1960</v>
+        <v>2852</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>2843</v>
+        <v>2853</v>
       </c>
       <c r="B251" t="s">
-        <v>1962</v>
+        <v>2854</v>
       </c>
       <c r="C251" t="s">
-        <v>1963</v>
+        <v>2855</v>
       </c>
       <c r="D251" t="s">
-        <v>1964</v>
+        <v>2856</v>
       </c>
       <c r="E251" t="s">
-        <v>1965</v>
+        <v>2857</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>2844</v>
+        <v>2862</v>
       </c>
       <c r="B252" t="s">
-        <v>2845</v>
+        <v>1977</v>
       </c>
       <c r="C252" t="s">
-        <v>1968</v>
+        <v>1976</v>
       </c>
       <c r="D252" t="s">
-        <v>1969</v>
+        <v>1978</v>
       </c>
       <c r="E252" t="s">
-        <v>1970</v>
+        <v>2867</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>2846</v>
+        <v>2868</v>
       </c>
       <c r="B253" t="s">
-        <v>2847</v>
+        <v>2869</v>
       </c>
       <c r="C253" t="s">
-        <v>2847</v>
+        <v>2870</v>
       </c>
       <c r="D253" t="s">
-        <v>2847</v>
+        <v>2871</v>
       </c>
       <c r="E253" t="s">
-        <v>2847</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>2848</v>
+        <v>2873</v>
       </c>
       <c r="B254" t="s">
-        <v>2849</v>
+        <v>2874</v>
       </c>
       <c r="C254" t="s">
-        <v>2850</v>
+        <v>2875</v>
       </c>
       <c r="D254" t="s">
-        <v>2851</v>
+        <v>2874</v>
       </c>
       <c r="E254" t="s">
-        <v>2852</v>
+        <v>2875</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>2853</v>
+        <v>2876</v>
       </c>
       <c r="B255" t="s">
-        <v>2854</v>
+        <v>2877</v>
       </c>
       <c r="C255" t="s">
-        <v>2855</v>
+        <v>2878</v>
       </c>
       <c r="D255" t="s">
-        <v>2856</v>
+        <v>2879</v>
       </c>
       <c r="E255" t="s">
-        <v>2857</v>
+        <v>2880</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>2862</v>
+        <v>2881</v>
       </c>
       <c r="B256" t="s">
-        <v>1977</v>
+        <v>2882</v>
       </c>
       <c r="C256" t="s">
-        <v>1976</v>
+        <v>2883</v>
       </c>
       <c r="D256" t="s">
-        <v>1978</v>
+        <v>2884</v>
       </c>
       <c r="E256" t="s">
-        <v>2867</v>
+        <v>2885</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>2868</v>
+        <v>2886</v>
       </c>
       <c r="B257" t="s">
-        <v>2869</v>
+        <v>2887</v>
       </c>
       <c r="C257" t="s">
-        <v>2870</v>
+        <v>2888</v>
       </c>
       <c r="D257" t="s">
-        <v>2871</v>
+        <v>2889</v>
       </c>
       <c r="E257" t="s">
-        <v>2872</v>
+        <v>2890</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>2873</v>
+        <v>2891</v>
       </c>
       <c r="B258" t="s">
-        <v>2874</v>
+        <v>2892</v>
       </c>
       <c r="C258" t="s">
-        <v>2875</v>
+        <v>2893</v>
       </c>
       <c r="D258" t="s">
-        <v>2874</v>
+        <v>2894</v>
       </c>
       <c r="E258" t="s">
-        <v>2875</v>
+        <v>2895</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>2876</v>
+        <v>2896</v>
       </c>
       <c r="B259" t="s">
-        <v>2877</v>
+        <v>2897</v>
       </c>
       <c r="C259" t="s">
-        <v>2878</v>
+        <v>2898</v>
       </c>
       <c r="D259" t="s">
-        <v>2879</v>
+        <v>2899</v>
       </c>
       <c r="E259" t="s">
-        <v>2880</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>2881</v>
+        <v>2901</v>
       </c>
       <c r="B260" t="s">
-        <v>2882</v>
+        <v>2902</v>
       </c>
       <c r="C260" t="s">
-        <v>2883</v>
+        <v>2903</v>
       </c>
       <c r="D260" t="s">
-        <v>2884</v>
+        <v>2904</v>
       </c>
       <c r="E260" t="s">
-        <v>2885</v>
+        <v>2905</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>2886</v>
+        <v>2906</v>
       </c>
       <c r="B261" t="s">
-        <v>2887</v>
+        <v>2907</v>
       </c>
       <c r="C261" t="s">
-        <v>2888</v>
+        <v>2908</v>
       </c>
       <c r="D261" t="s">
-        <v>2889</v>
+        <v>2909</v>
       </c>
       <c r="E261" t="s">
-        <v>2890</v>
+        <v>2910</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>2891</v>
+        <v>2911</v>
       </c>
       <c r="B262" t="s">
-        <v>2892</v>
+        <v>2912</v>
       </c>
       <c r="C262" t="s">
-        <v>2893</v>
+        <v>2913</v>
       </c>
       <c r="D262" t="s">
-        <v>2894</v>
+        <v>2914</v>
       </c>
       <c r="E262" t="s">
-        <v>2895</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>2896</v>
+        <v>2916</v>
       </c>
       <c r="B263" t="s">
-        <v>2897</v>
+        <v>2917</v>
       </c>
       <c r="C263" t="s">
-        <v>2898</v>
+        <v>2918</v>
       </c>
       <c r="D263" t="s">
-        <v>2899</v>
+        <v>2919</v>
       </c>
       <c r="E263" t="s">
-        <v>2900</v>
+        <v>2920</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>2901</v>
+        <v>2921</v>
       </c>
       <c r="B264" t="s">
-        <v>2902</v>
+        <v>2922</v>
       </c>
       <c r="C264" t="s">
-        <v>2903</v>
+        <v>2923</v>
       </c>
       <c r="D264" t="s">
-        <v>2904</v>
+        <v>2924</v>
       </c>
       <c r="E264" t="s">
-        <v>2905</v>
+        <v>2925</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>2906</v>
+        <v>2928</v>
       </c>
       <c r="B265" t="s">
-        <v>2907</v>
+        <v>2929</v>
       </c>
       <c r="C265" t="s">
-        <v>2908</v>
+        <v>2930</v>
       </c>
       <c r="D265" t="s">
-        <v>2909</v>
+        <v>2931</v>
       </c>
       <c r="E265" t="s">
-        <v>2910</v>
+        <v>2932</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>2911</v>
+        <v>2933</v>
       </c>
       <c r="B266" t="s">
-        <v>2912</v>
+        <v>2934</v>
       </c>
       <c r="C266" t="s">
-        <v>2913</v>
+        <v>2935</v>
       </c>
       <c r="D266" t="s">
-        <v>2914</v>
+        <v>2936</v>
       </c>
       <c r="E266" t="s">
-        <v>2915</v>
+        <v>2937</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>2916</v>
+        <v>2938</v>
       </c>
       <c r="B267" t="s">
-        <v>2917</v>
+        <v>2939</v>
       </c>
       <c r="C267" t="s">
-        <v>2918</v>
+        <v>2940</v>
       </c>
       <c r="D267" t="s">
-        <v>2919</v>
+        <v>2941</v>
       </c>
       <c r="E267" t="s">
-        <v>2920</v>
+        <v>2942</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="s">
+        <v>2943</v>
+      </c>
+      <c r="B268" t="s">
+        <v>2944</v>
+      </c>
+      <c r="C268" t="s">
+        <v>2945</v>
+      </c>
+      <c r="D268" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E268" t="s">
+        <v>2947</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="s">
+        <v>2948</v>
+      </c>
+      <c r="B269" t="s">
+        <v>2949</v>
+      </c>
+      <c r="C269" t="s">
+        <v>2950</v>
+      </c>
+      <c r="D269" t="s">
+        <v>2951</v>
+      </c>
+      <c r="E269" t="s">
+        <v>2952</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="s">
+        <v>2958</v>
+      </c>
+      <c r="B270" t="s">
+        <v>2808</v>
+      </c>
+      <c r="C270" t="s">
+        <v>2809</v>
+      </c>
+      <c r="D270" t="s">
+        <v>2959</v>
+      </c>
+      <c r="E270" t="s">
+        <v>2811</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="s">
+        <v>2960</v>
+      </c>
+      <c r="B271" t="s">
+        <v>2961</v>
+      </c>
+      <c r="C271" t="s">
+        <v>2962</v>
+      </c>
+      <c r="D271" t="s">
+        <v>2963</v>
+      </c>
+      <c r="E271" t="s">
+        <v>2964</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="s">
+        <v>2965</v>
+      </c>
+      <c r="B272" t="s">
+        <v>2966</v>
+      </c>
+      <c r="C272" t="s">
+        <v>2967</v>
+      </c>
+      <c r="D272" t="s">
+        <v>2968</v>
+      </c>
+      <c r="E272" t="s">
+        <v>2969</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="s">
+        <v>2970</v>
+      </c>
+      <c r="B273" t="s">
+        <v>2971</v>
+      </c>
+      <c r="C273" t="s">
+        <v>2972</v>
+      </c>
+      <c r="D273" t="s">
+        <v>2973</v>
+      </c>
+      <c r="E273" t="s">
+        <v>2974</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="s">
+        <v>2975</v>
+      </c>
+      <c r="B274" t="s">
+        <v>2976</v>
+      </c>
+      <c r="C274" t="s">
+        <v>2977</v>
+      </c>
+      <c r="D274" t="s">
+        <v>2978</v>
+      </c>
+      <c r="E274" t="s">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="s">
+        <v>2980</v>
+      </c>
+      <c r="B275" t="s">
+        <v>2981</v>
+      </c>
+      <c r="C275" t="s">
+        <v>2982</v>
+      </c>
+      <c r="D275" t="s">
+        <v>2983</v>
+      </c>
+      <c r="E275" t="s">
+        <v>2984</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="s">
+        <v>2985</v>
+      </c>
+      <c r="B276" t="s">
+        <v>2986</v>
+      </c>
+      <c r="C276" t="s">
+        <v>2987</v>
+      </c>
+      <c r="D276" t="s">
+        <v>2988</v>
+      </c>
+      <c r="E276" t="s">
+        <v>2989</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="s">
+        <v>2953</v>
+      </c>
+      <c r="B277" t="s">
+        <v>2990</v>
+      </c>
+      <c r="C277" t="s">
+        <v>2991</v>
+      </c>
+      <c r="D277" t="s">
+        <v>2992</v>
+      </c>
+      <c r="E277" t="s">
+        <v>2993</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="s">
+        <v>2994</v>
+      </c>
+      <c r="B278" t="s">
+        <v>2995</v>
+      </c>
+      <c r="C278" t="s">
+        <v>2996</v>
+      </c>
+      <c r="D278" t="s">
+        <v>2997</v>
+      </c>
+      <c r="E278" t="s">
+        <v>2998</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="s">
+        <v>3003</v>
+      </c>
+      <c r="B279" t="s">
+        <v>3004</v>
+      </c>
+      <c r="C279" t="s">
+        <v>3005</v>
+      </c>
+      <c r="D279" t="s">
+        <v>3006</v>
+      </c>
+      <c r="E279" t="s">
+        <v>3007</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="s">
+        <v>3008</v>
+      </c>
+      <c r="B280" t="s">
+        <v>2647</v>
+      </c>
+      <c r="C280" t="s">
+        <v>2648</v>
+      </c>
+      <c r="D280" t="s">
+        <v>2647</v>
+      </c>
+      <c r="E280" t="s">
+        <v>3009</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="s">
+        <v>3010</v>
+      </c>
+      <c r="B281" t="s">
+        <v>3011</v>
+      </c>
+      <c r="C281" t="s">
+        <v>3012</v>
+      </c>
+      <c r="D281" t="s">
+        <v>3013</v>
+      </c>
+      <c r="E281" t="s">
+        <v>3014</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="s">
+        <v>3015</v>
+      </c>
+      <c r="B282" t="s">
+        <v>3016</v>
+      </c>
+      <c r="C282" t="s">
+        <v>3017</v>
+      </c>
+      <c r="D282" t="s">
+        <v>3018</v>
+      </c>
+      <c r="E282" t="s">
+        <v>3019</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="s">
+        <v>3020</v>
+      </c>
+      <c r="B283" t="s">
+        <v>3021</v>
+      </c>
+      <c r="C283" t="s">
+        <v>3022</v>
+      </c>
+      <c r="D283" t="s">
+        <v>3023</v>
+      </c>
+      <c r="E283" t="s">
+        <v>3024</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="s">
+        <v>3025</v>
+      </c>
+      <c r="B284" t="s">
+        <v>3026</v>
+      </c>
+      <c r="C284" t="s">
+        <v>3027</v>
+      </c>
+      <c r="D284" t="s">
+        <v>3028</v>
+      </c>
+      <c r="E284" t="s">
+        <v>3029</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="s">
+        <v>3030</v>
+      </c>
+      <c r="B285" t="s">
+        <v>1856</v>
+      </c>
+      <c r="C285" t="s">
+        <v>1857</v>
+      </c>
+      <c r="D285" t="s">
+        <v>1858</v>
+      </c>
+      <c r="E285" t="s">
+        <v>3031</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="s">
+        <v>3044</v>
+      </c>
+      <c r="B286" t="s">
+        <v>3045</v>
+      </c>
+      <c r="C286" t="s">
+        <v>3046</v>
+      </c>
+      <c r="D286" t="s">
+        <v>3047</v>
+      </c>
+      <c r="E286" t="s">
+        <v>3048</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="s">
+        <v>3049</v>
+      </c>
+      <c r="B287" t="s">
+        <v>3050</v>
+      </c>
+      <c r="C287" t="s">
+        <v>3051</v>
+      </c>
+      <c r="D287" t="s">
+        <v>3052</v>
+      </c>
+      <c r="E287" t="s">
+        <v>3053</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="s">
+        <v>3054</v>
+      </c>
+      <c r="B288" t="s">
+        <v>3055</v>
+      </c>
+      <c r="C288" t="s">
+        <v>3056</v>
+      </c>
+      <c r="D288" t="s">
+        <v>3057</v>
+      </c>
+      <c r="E288" t="s">
+        <v>3058</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="s">
+        <v>3059</v>
+      </c>
+      <c r="B289" t="s">
+        <v>3060</v>
+      </c>
+      <c r="C289" t="s">
+        <v>3061</v>
+      </c>
+      <c r="D289" t="s">
+        <v>3062</v>
+      </c>
+      <c r="E289" t="s">
+        <v>3063</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="s">
+        <v>3064</v>
+      </c>
+      <c r="B290" t="s">
+        <v>3065</v>
+      </c>
+      <c r="C290" t="s">
+        <v>3066</v>
+      </c>
+      <c r="D290" t="s">
+        <v>3067</v>
+      </c>
+      <c r="E290" t="s">
+        <v>3068</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="s">
+        <v>3069</v>
+      </c>
+      <c r="B291" t="s">
+        <v>3070</v>
+      </c>
+      <c r="C291" t="s">
+        <v>3071</v>
+      </c>
+      <c r="D291" t="s">
+        <v>3072</v>
+      </c>
+      <c r="E291" t="s">
+        <v>3073</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="s">
+        <v>3074</v>
+      </c>
+      <c r="B292" t="s">
+        <v>1985</v>
+      </c>
+      <c r="C292" t="s">
+        <v>1986</v>
+      </c>
+      <c r="D292" t="s">
+        <v>1987</v>
+      </c>
+      <c r="E292" t="s">
+        <v>1988</v>
       </c>
     </row>
   </sheetData>

</xml_diff>